<commit_message>
docs(audit): reconcile audit reports and closeout spec with honest evidence and PO approval gates
</commit_message>
<xml_diff>
--- a/docs/plans/Digiwin_Semiconductor_Theo_doi_ngan_sach.xlsx
+++ b/docs/plans/Digiwin_Semiconductor_Theo_doi_ngan_sach.xlsx
@@ -2159,7 +2159,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -2905,7 +2904,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -3536,8 +3534,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -23475,7 +23471,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="107" t="inlineStr">
         <is>
@@ -23566,12 +23561,12 @@
       </c>
       <c r="G5" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H5" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I5" s="141" t="inlineStr">
@@ -23623,12 +23618,12 @@
       </c>
       <c r="G6" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H6" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I6" s="141" t="inlineStr">
@@ -23680,12 +23675,12 @@
       </c>
       <c r="G7" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H7" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I7" s="141" t="inlineStr">
@@ -23737,12 +23732,12 @@
       </c>
       <c r="G8" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H8" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I8" s="141" t="inlineStr">
@@ -23794,12 +23789,12 @@
       </c>
       <c r="G9" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H9" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I9" s="141" t="inlineStr">
@@ -23851,12 +23846,12 @@
       </c>
       <c r="G10" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H10" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I10" s="141" t="inlineStr">
@@ -23908,12 +23903,12 @@
       </c>
       <c r="G11" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H11" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I11" s="141" t="inlineStr">
@@ -23965,12 +23960,12 @@
       </c>
       <c r="G12" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H12" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I12" s="141" t="inlineStr">
@@ -24022,12 +24017,12 @@
       </c>
       <c r="G13" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H13" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I13" s="141" t="inlineStr">
@@ -24079,12 +24074,12 @@
       </c>
       <c r="G14" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H14" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I14" s="141" t="inlineStr">
@@ -24136,12 +24131,12 @@
       </c>
       <c r="G15" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H15" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I15" s="141" t="inlineStr">
@@ -24193,12 +24188,12 @@
       </c>
       <c r="G16" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H16" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I16" s="141" t="inlineStr">
@@ -24250,12 +24245,12 @@
       </c>
       <c r="G17" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H17" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I17" s="141" t="inlineStr">
@@ -24307,12 +24302,12 @@
       </c>
       <c r="G18" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H18" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I18" s="141" t="inlineStr">
@@ -24364,12 +24359,12 @@
       </c>
       <c r="G19" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H19" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I19" s="141" t="inlineStr">
@@ -24421,12 +24416,12 @@
       </c>
       <c r="G20" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H20" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I20" s="141" t="inlineStr">
@@ -24478,12 +24473,12 @@
       </c>
       <c r="G21" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H21" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I21" s="141" t="inlineStr">
@@ -24535,12 +24530,12 @@
       </c>
       <c r="G22" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H22" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I22" s="141" t="inlineStr">
@@ -24592,12 +24587,12 @@
       </c>
       <c r="G23" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H23" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I23" s="141" t="inlineStr">
@@ -24649,12 +24644,12 @@
       </c>
       <c r="G24" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H24" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I24" s="141" t="inlineStr">
@@ -24706,12 +24701,12 @@
       </c>
       <c r="G25" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H25" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I25" s="141" t="inlineStr">
@@ -24763,12 +24758,12 @@
       </c>
       <c r="G26" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H26" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I26" s="141" t="inlineStr">
@@ -24820,12 +24815,12 @@
       </c>
       <c r="G27" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H27" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I27" s="141" t="inlineStr">
@@ -24877,12 +24872,12 @@
       </c>
       <c r="G28" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H28" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I28" s="141" t="inlineStr">
@@ -24934,12 +24929,12 @@
       </c>
       <c r="G29" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H29" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I29" s="141" t="inlineStr">
@@ -24991,12 +24986,12 @@
       </c>
       <c r="G30" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H30" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I30" s="141" t="inlineStr">
@@ -25048,12 +25043,12 @@
       </c>
       <c r="G31" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H31" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I31" s="141" t="inlineStr">
@@ -25105,12 +25100,12 @@
       </c>
       <c r="G32" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H32" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I32" s="141" t="inlineStr">
@@ -25132,7 +25127,7 @@
     <row r="33">
       <c r="A33" s="141" t="inlineStr">
         <is>
-          <t>Keyword (Observed)</t>
+          <t>Observed query (EN)</t>
         </is>
       </c>
       <c r="B33" s="142" t="inlineStr">
@@ -25147,7 +25142,7 @@
       </c>
       <c r="D33" s="142" t="inlineStr">
         <is>
-          <t>Solution</t>
+          <t>Solution (ERP partner)</t>
         </is>
       </c>
       <c r="E33" s="142" t="inlineStr">
@@ -25157,17 +25152,15 @@
       </c>
       <c r="F33" s="141" t="inlineStr">
         <is>
-          <t>Phrase</t>
-        </is>
-      </c>
-      <c r="G33" s="143" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+          <t>Historical observation</t>
+        </is>
+      </c>
+      <c r="G33" s="143" t="n">
+        <v>10</v>
       </c>
       <c r="H33" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Vietnam, Vietnamese, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I33" s="141" t="inlineStr">
@@ -25177,7 +25170,7 @@
       </c>
       <c r="J33" s="141" t="inlineStr">
         <is>
-          <t>Quan sát Keyword Planner</t>
+          <t>Verified historical observation; 3-mo change 0%, YoY -100%</t>
         </is>
       </c>
       <c r="K33" s="142" t="inlineStr">
@@ -25219,12 +25212,12 @@
       </c>
       <c r="G34" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H34" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I34" s="141" t="inlineStr">
@@ -25234,7 +25227,7 @@
       </c>
       <c r="J34" s="141" t="inlineStr">
         <is>
-          <t>Brand candidate</t>
+          <t>Brand candidate; chưa query</t>
         </is>
       </c>
       <c r="K34" s="142" t="inlineStr">
@@ -25276,12 +25269,12 @@
       </c>
       <c r="G35" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H35" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I35" s="141" t="inlineStr">
@@ -25291,7 +25284,7 @@
       </c>
       <c r="J35" s="141" t="inlineStr">
         <is>
-          <t>Brand candidate</t>
+          <t>Brand candidate; chưa query</t>
         </is>
       </c>
       <c r="K35" s="142" t="inlineStr">
@@ -25333,12 +25326,12 @@
       </c>
       <c r="G36" s="143" t="inlineStr">
         <is>
-          <t>- (no displayed data)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H36" s="142" t="inlineStr">
         <is>
-          <t>Vietnam, Sep 2025-Aug 2026</t>
+          <t>Not queried</t>
         </is>
       </c>
       <c r="I36" s="141" t="inlineStr">
@@ -25348,7 +25341,7 @@
       </c>
       <c r="J36" s="141" t="inlineStr">
         <is>
-          <t>Brand candidate</t>
+          <t>Brand candidate; chưa query</t>
         </is>
       </c>
       <c r="K36" s="142" t="inlineStr">
@@ -25390,22 +25383,22 @@
       </c>
       <c r="G37" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H37" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I37" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J37" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K37" s="142" t="inlineStr">
@@ -25447,22 +25440,22 @@
       </c>
       <c r="G38" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H38" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I38" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J38" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K38" s="142" t="inlineStr">
@@ -25504,22 +25497,22 @@
       </c>
       <c r="G39" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H39" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I39" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J39" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K39" s="142" t="inlineStr">
@@ -25561,22 +25554,22 @@
       </c>
       <c r="G40" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H40" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I40" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J40" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K40" s="142" t="inlineStr">
@@ -25618,22 +25611,22 @@
       </c>
       <c r="G41" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H41" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I41" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J41" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K41" s="142" t="inlineStr">
@@ -25675,22 +25668,22 @@
       </c>
       <c r="G42" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H42" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I42" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J42" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K42" s="142" t="inlineStr">
@@ -25732,22 +25725,22 @@
       </c>
       <c r="G43" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H43" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I43" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J43" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K43" s="142" t="inlineStr">
@@ -25789,22 +25782,22 @@
       </c>
       <c r="G44" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H44" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I44" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J44" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K44" s="142" t="inlineStr">
@@ -25846,22 +25839,22 @@
       </c>
       <c r="G45" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H45" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I45" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J45" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K45" s="142" t="inlineStr">
@@ -25903,22 +25896,22 @@
       </c>
       <c r="G46" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H46" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I46" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J46" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K46" s="142" t="inlineStr">
@@ -25960,22 +25953,22 @@
       </c>
       <c r="G47" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H47" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I47" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J47" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K47" s="142" t="inlineStr">
@@ -26017,22 +26010,22 @@
       </c>
       <c r="G48" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H48" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I48" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J48" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K48" s="142" t="inlineStr">
@@ -26074,22 +26067,22 @@
       </c>
       <c r="G49" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H49" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I49" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J49" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K49" s="142" t="inlineStr">
@@ -26131,22 +26124,22 @@
       </c>
       <c r="G50" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H50" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I50" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J50" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K50" s="142" t="inlineStr">
@@ -26188,22 +26181,22 @@
       </c>
       <c r="G51" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H51" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I51" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J51" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K51" s="142" t="inlineStr">
@@ -26245,22 +26238,22 @@
       </c>
       <c r="G52" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H52" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I52" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J52" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K52" s="142" t="inlineStr">
@@ -26302,22 +26295,22 @@
       </c>
       <c r="G53" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H53" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I53" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J53" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K53" s="142" t="inlineStr">
@@ -26359,22 +26352,22 @@
       </c>
       <c r="G54" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H54" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I54" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J54" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K54" s="142" t="inlineStr">
@@ -26416,22 +26409,22 @@
       </c>
       <c r="G55" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H55" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I55" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J55" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K55" s="142" t="inlineStr">
@@ -26473,22 +26466,22 @@
       </c>
       <c r="G56" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H56" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I56" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J56" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K56" s="142" t="inlineStr">
@@ -26530,22 +26523,22 @@
       </c>
       <c r="G57" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H57" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I57" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J57" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K57" s="142" t="inlineStr">
@@ -26587,22 +26580,22 @@
       </c>
       <c r="G58" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H58" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I58" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J58" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K58" s="142" t="inlineStr">
@@ -26644,22 +26637,22 @@
       </c>
       <c r="G59" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H59" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I59" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J59" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K59" s="142" t="inlineStr">
@@ -26701,22 +26694,22 @@
       </c>
       <c r="G60" s="143" t="inlineStr">
         <is>
-          <t>- (negative)</t>
+          <t>N/A (Negative)</t>
         </is>
       </c>
       <c r="H60" s="142" t="inlineStr">
         <is>
-          <t>Toàn quốc</t>
+          <t>Negative list review</t>
         </is>
       </c>
       <c r="I60" s="141" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J60" s="141" t="inlineStr">
         <is>
-          <t>Chưa áp dụng</t>
+          <t>Candidate negative keyword</t>
         </is>
       </c>
       <c r="K60" s="142" t="inlineStr">

</xml_diff>

<commit_message>
feat(search): record Codex Google Keyword Planner multilingual discovery receipt, evidence and audit report
</commit_message>
<xml_diff>
--- a/docs/plans/Digiwin_Semiconductor_Theo_doi_ngan_sach.xlsx
+++ b/docs/plans/Digiwin_Semiconductor_Theo_doi_ngan_sach.xlsx
@@ -23960,17 +23960,17 @@
       </c>
       <c r="G12" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H12" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, English, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I12" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J12" s="141" t="inlineStr">
@@ -24017,17 +24017,17 @@
       </c>
       <c r="G13" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H13" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, English, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I13" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J13" s="141" t="inlineStr">
@@ -24074,17 +24074,17 @@
       </c>
       <c r="G14" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H14" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, English, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I14" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J14" s="141" t="inlineStr">
@@ -24131,17 +24131,17 @@
       </c>
       <c r="G15" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H15" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, English, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I15" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J15" s="141" t="inlineStr">
@@ -24188,17 +24188,17 @@
       </c>
       <c r="G16" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H16" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, English, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I16" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J16" s="141" t="inlineStr">
@@ -24245,17 +24245,17 @@
       </c>
       <c r="G17" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H17" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, English, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I17" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J17" s="141" t="inlineStr">
@@ -24302,17 +24302,17 @@
       </c>
       <c r="G18" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H18" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, English, Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I18" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J18" s="141" t="inlineStr">
@@ -24359,17 +24359,17 @@
       </c>
       <c r="G19" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H19" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (simplified), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I19" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J19" s="141" t="inlineStr">
@@ -24416,17 +24416,17 @@
       </c>
       <c r="G20" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H20" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (simplified), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I20" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J20" s="141" t="inlineStr">
@@ -24473,17 +24473,17 @@
       </c>
       <c r="G21" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H21" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (simplified), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I21" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J21" s="141" t="inlineStr">
@@ -24530,17 +24530,17 @@
       </c>
       <c r="G22" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H22" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (simplified), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I22" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J22" s="141" t="inlineStr">
@@ -24587,17 +24587,17 @@
       </c>
       <c r="G23" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H23" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (simplified), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I23" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J23" s="141" t="inlineStr">
@@ -24644,17 +24644,17 @@
       </c>
       <c r="G24" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H24" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (simplified), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I24" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J24" s="141" t="inlineStr">
@@ -24701,17 +24701,17 @@
       </c>
       <c r="G25" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H25" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (simplified), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I25" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J25" s="141" t="inlineStr">
@@ -24758,17 +24758,17 @@
       </c>
       <c r="G26" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H26" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (traditional), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I26" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J26" s="141" t="inlineStr">
@@ -24815,17 +24815,17 @@
       </c>
       <c r="G27" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H27" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (traditional), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I27" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J27" s="141" t="inlineStr">
@@ -24872,17 +24872,17 @@
       </c>
       <c r="G28" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H28" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (traditional), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I28" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J28" s="141" t="inlineStr">
@@ -24929,17 +24929,17 @@
       </c>
       <c r="G29" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H29" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (traditional), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I29" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J29" s="141" t="inlineStr">
@@ -24986,17 +24986,17 @@
       </c>
       <c r="G30" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H30" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (traditional), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I30" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J30" s="141" t="inlineStr">
@@ -25043,17 +25043,17 @@
       </c>
       <c r="G31" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H31" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (traditional), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I31" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J31" s="141" t="inlineStr">
@@ -25100,17 +25100,17 @@
       </c>
       <c r="G32" s="143" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H32" s="142" t="inlineStr">
         <is>
-          <t>Not queried</t>
+          <t>Vietnam, Chinese (traditional), Sep 2025-Aug 2026</t>
         </is>
       </c>
       <c r="I32" s="141" t="inlineStr">
         <is>
-          <t>Chưa query</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J32" s="141" t="inlineStr">

</xml_diff>